<commit_message>
Add RMT automation framework with safe runtime configuration
</commit_message>
<xml_diff>
--- a/src/test/TestData/Designation Master.xlsx
+++ b/src/test/TestData/Designation Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Piyush.Wadhwa\IdeaProjects\Automation\RMT\src\test\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2052208A-D4FC-4C55-BD7A-CCF56FBE8E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CAB125-E6E2-412E-A7A4-185330CDB570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Designation Master" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Designation Master'!$A$1:$M$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Designation Master'!$A$1:$M$138</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1726" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1674" uniqueCount="648">
   <si>
     <t>DESGN_ID</t>
   </si>
@@ -1853,82 +1853,133 @@
     <t>//li[text()='Clients &amp; Markets Leader - Advisory Services']</t>
   </si>
   <si>
-    <t>//li[text()='Partner and Leader – Private Client Services']</t>
-  </si>
-  <si>
-    <t>//li[text()='Partner &amp; COO']</t>
-  </si>
-  <si>
-    <t>//li[text()='Partner – National Management']</t>
-  </si>
-  <si>
-    <t>ASSISTANT MANAGER WINGS</t>
-  </si>
-  <si>
-    <t>ASSOCIATE DIRECTOR WINGS</t>
-  </si>
-  <si>
-    <t>CONSULTANT WINGS</t>
-  </si>
-  <si>
-    <t>CSS4 WINGS</t>
-  </si>
-  <si>
-    <t>//li[text()='CSS4 WINGS']</t>
-  </si>
-  <si>
-    <t>DIRECTOR WINGS</t>
-  </si>
-  <si>
-    <t>DIRECTOR – IKCC</t>
-  </si>
-  <si>
-    <t>EXECUTIVE DIRECTOR WINGS</t>
-  </si>
-  <si>
-    <t>MANAGER WINGS</t>
-  </si>
-  <si>
-    <t>PARTNER - CLIENTS &amp; MARKETS</t>
-  </si>
-  <si>
-    <t>PARTNER-WINGS</t>
-  </si>
-  <si>
-    <t>RMS TESTING</t>
-  </si>
-  <si>
-    <t>TRAINEE WINGS</t>
-  </si>
-  <si>
-    <t>//li[text()='Assistant Manager WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Associate Director WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Consultant WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Director WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Director – IKCC']</t>
-  </si>
-  <si>
-    <t>//li[text()='Executive Director WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Manager WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Partner-WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Trainee WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='RMS Testing']</t>
+    <t>US000013</t>
+  </si>
+  <si>
+    <t>US000002</t>
+  </si>
+  <si>
+    <t>04-OCT-11</t>
+  </si>
+  <si>
+    <t>08-NOV-25</t>
+  </si>
+  <si>
+    <t>US000014</t>
+  </si>
+  <si>
+    <t>US000003</t>
+  </si>
+  <si>
+    <t>04-OCT-12</t>
+  </si>
+  <si>
+    <t>08-NOV-26</t>
+  </si>
+  <si>
+    <t>US000015</t>
+  </si>
+  <si>
+    <t>US000004</t>
+  </si>
+  <si>
+    <t>04-OCT-13</t>
+  </si>
+  <si>
+    <t>08-NOV-27</t>
+  </si>
+  <si>
+    <t>US000016</t>
+  </si>
+  <si>
+    <t>US000005</t>
+  </si>
+  <si>
+    <t>04-OCT-14</t>
+  </si>
+  <si>
+    <t>08-NOV-28</t>
+  </si>
+  <si>
+    <t>US000017</t>
+  </si>
+  <si>
+    <t>US000006</t>
+  </si>
+  <si>
+    <t>04-OCT-15</t>
+  </si>
+  <si>
+    <t>08-NOV-29</t>
+  </si>
+  <si>
+    <t>US000018</t>
+  </si>
+  <si>
+    <t>US000007</t>
+  </si>
+  <si>
+    <t>04-OCT-16</t>
+  </si>
+  <si>
+    <t>08-NOV-30</t>
+  </si>
+  <si>
+    <t>US000019</t>
+  </si>
+  <si>
+    <t>US000008</t>
+  </si>
+  <si>
+    <t>04-OCT-17</t>
+  </si>
+  <si>
+    <t>08-NOV-31</t>
+  </si>
+  <si>
+    <t>US000020</t>
+  </si>
+  <si>
+    <t>US000009</t>
+  </si>
+  <si>
+    <t>04-OCT-18</t>
+  </si>
+  <si>
+    <t>08-NOV-32</t>
+  </si>
+  <si>
+    <t>//li[text()='Associate Consultant']</t>
+  </si>
+  <si>
+    <t>//li[text()='Change Management Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Chief Information Officer']</t>
+  </si>
+  <si>
+    <t>//li[text()='Client Experience Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner,CPCO']</t>
+  </si>
+  <si>
+    <t>//li[text()='Strategic Sourcing Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Transformation &amp; Innovation Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Travel Incharge - Office of the CEO']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner, COO']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner - National Managementment']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner and Leader - Private Client Services']</t>
   </si>
 </sst>
 </file>
@@ -1952,7 +2003,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2031,7 +2082,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2049,34 +2100,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2417,10 +2460,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M142"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.77734375" customWidth="1"/>
@@ -2432,7 +2475,7 @@
     <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16.88671875" customWidth="1"/>
-    <col min="10" max="10" width="68.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="68.77734375" style="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -2466,7 +2509,7 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="7" t="s">
         <v>469</v>
       </c>
       <c r="K1" s="2" t="s">
@@ -2479,7 +2522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -2507,7 +2550,7 @@
       <c r="I2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="8" t="s">
         <v>593</v>
       </c>
       <c r="K2" s="1" t="s">
@@ -2544,7 +2587,7 @@
       <c r="I3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="8" t="s">
         <v>471</v>
       </c>
       <c r="K3" s="1" t="s">
@@ -2557,7 +2600,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
@@ -2585,7 +2628,7 @@
       <c r="I4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="8" t="s">
         <v>472</v>
       </c>
       <c r="K4" s="1" t="s">
@@ -2598,7 +2641,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
@@ -2626,7 +2669,7 @@
       <c r="I5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="8" t="s">
         <v>473</v>
       </c>
       <c r="K5" s="1" t="s">
@@ -2663,7 +2706,7 @@
       <c r="I6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="8" t="s">
         <v>476</v>
       </c>
       <c r="K6" s="1" t="s">
@@ -2704,7 +2747,7 @@
       <c r="I7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="8" t="s">
         <v>475</v>
       </c>
       <c r="K7" s="1" t="s">
@@ -2717,7 +2760,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>350</v>
       </c>
@@ -2741,7 +2784,7 @@
       <c r="I8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="8" t="s">
         <v>477</v>
       </c>
       <c r="K8" s="1" t="s">
@@ -2754,7 +2797,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
@@ -2782,7 +2825,7 @@
       <c r="I9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="8" t="s">
         <v>478</v>
       </c>
       <c r="K9" s="1" t="s">
@@ -2795,7 +2838,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>118</v>
       </c>
@@ -2823,7 +2866,7 @@
       <c r="I10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="8" t="s">
         <v>479</v>
       </c>
       <c r="K10" s="1" t="s">
@@ -2836,7 +2879,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>121</v>
       </c>
@@ -2864,7 +2907,7 @@
       <c r="I11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="8" t="s">
         <v>480</v>
       </c>
       <c r="K11" s="1" t="s">
@@ -2877,7 +2920,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>64</v>
       </c>
@@ -2905,7 +2948,7 @@
       <c r="I12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="8" t="s">
         <v>474</v>
       </c>
       <c r="K12" s="1" t="s">
@@ -2918,7 +2961,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>408</v>
       </c>
@@ -2946,7 +2989,7 @@
       <c r="I13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="8" t="s">
         <v>481</v>
       </c>
       <c r="K13" s="1" t="s">
@@ -2987,7 +3030,7 @@
       <c r="I14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="8" t="s">
         <v>482</v>
       </c>
       <c r="K14" s="1" t="s">
@@ -3000,7 +3043,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>115</v>
       </c>
@@ -3028,7 +3071,7 @@
       <c r="I15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="J15" s="8" t="s">
         <v>483</v>
       </c>
       <c r="K15" s="1" t="s">
@@ -3041,7 +3084,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>329</v>
       </c>
@@ -3065,7 +3108,7 @@
       <c r="I16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="J16" s="8" t="s">
         <v>484</v>
       </c>
       <c r="K16" s="1" t="s">
@@ -3078,7 +3121,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>209</v>
       </c>
@@ -3106,7 +3149,7 @@
       <c r="I17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="8" t="s">
         <v>485</v>
       </c>
       <c r="K17" s="1" t="s">
@@ -3143,7 +3186,7 @@
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="8" t="s">
         <v>486</v>
       </c>
       <c r="K18" s="1" t="s">
@@ -3180,7 +3223,7 @@
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="J19" s="8" t="s">
         <v>488</v>
       </c>
       <c r="K19" s="1" t="s">
@@ -3193,7 +3236,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>284</v>
       </c>
@@ -3217,7 +3260,7 @@
       <c r="I20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="1" t="s">
+      <c r="J20" s="8" t="s">
         <v>489</v>
       </c>
       <c r="K20" s="1" t="s">
@@ -3230,7 +3273,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>381</v>
       </c>
@@ -3254,7 +3297,7 @@
       <c r="I21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="J21" s="8" t="s">
         <v>491</v>
       </c>
       <c r="K21" s="1" t="s">
@@ -3267,7 +3310,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>375</v>
       </c>
@@ -3291,7 +3334,7 @@
       <c r="I22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="J22" s="8" t="s">
         <v>487</v>
       </c>
       <c r="K22" s="1" t="s">
@@ -3328,7 +3371,7 @@
       <c r="I23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="J23" s="8" t="s">
         <v>490</v>
       </c>
       <c r="K23" s="1" t="s">
@@ -3341,7 +3384,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>392</v>
       </c>
@@ -3365,7 +3408,7 @@
       <c r="I24" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="J24" s="8" t="s">
         <v>493</v>
       </c>
       <c r="K24" s="1" t="s">
@@ -3402,7 +3445,7 @@
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J25" s="1" t="s">
+      <c r="J25" s="8" t="s">
         <v>494</v>
       </c>
       <c r="K25" s="1" t="s">
@@ -3415,7 +3458,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>396</v>
       </c>
@@ -3439,7 +3482,7 @@
       <c r="I26" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="J26" s="8" t="s">
         <v>492</v>
       </c>
       <c r="K26" s="1" t="s">
@@ -3452,7 +3495,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>49</v>
       </c>
@@ -3480,7 +3523,7 @@
       <c r="I27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J27" s="1" t="s">
+      <c r="J27" s="8" t="s">
         <v>495</v>
       </c>
       <c r="K27" s="1" t="s">
@@ -3493,7 +3536,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>146</v>
       </c>
@@ -3517,7 +3560,7 @@
       <c r="I28" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J28" s="1" t="s">
+      <c r="J28" s="8" t="s">
         <v>496</v>
       </c>
       <c r="K28" s="1" t="s">
@@ -3530,7 +3573,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>366</v>
       </c>
@@ -3554,7 +3597,7 @@
       <c r="I29" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="J29" s="8" t="s">
         <v>497</v>
       </c>
       <c r="K29" s="1" t="s">
@@ -3567,7 +3610,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>419</v>
       </c>
@@ -3591,7 +3634,7 @@
       <c r="I30" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="J30" s="8" t="s">
         <v>498</v>
       </c>
       <c r="K30" s="1" t="s">
@@ -3604,7 +3647,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>356</v>
       </c>
@@ -3628,7 +3671,7 @@
       <c r="I31" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="J31" s="8" t="s">
         <v>499</v>
       </c>
       <c r="K31" s="1" t="s">
@@ -3641,7 +3684,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>347</v>
       </c>
@@ -3665,7 +3708,7 @@
       <c r="I32" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="J32" s="8" t="s">
         <v>500</v>
       </c>
       <c r="K32" s="1" t="s">
@@ -3678,7 +3721,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>369</v>
       </c>
@@ -3702,7 +3745,7 @@
       <c r="I33" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="J33" s="8" t="s">
         <v>502</v>
       </c>
       <c r="K33" s="1" t="s">
@@ -3715,7 +3758,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>300</v>
       </c>
@@ -3739,7 +3782,7 @@
       <c r="I34" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="J34" s="8" t="s">
         <v>501</v>
       </c>
       <c r="K34" s="1" t="s">
@@ -3752,7 +3795,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>343</v>
       </c>
@@ -3776,7 +3819,7 @@
       <c r="I35" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="J35" s="8" t="s">
         <v>503</v>
       </c>
       <c r="K35" s="1" t="s">
@@ -3789,7 +3832,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>416</v>
       </c>
@@ -3813,7 +3856,7 @@
       <c r="I36" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="J36" s="8" t="s">
         <v>504</v>
       </c>
       <c r="K36" s="1" t="s">
@@ -3826,7 +3869,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>291</v>
       </c>
@@ -3850,7 +3893,7 @@
       <c r="I37" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="J37" s="8" t="s">
         <v>505</v>
       </c>
       <c r="K37" s="1" t="s">
@@ -3863,7 +3906,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>372</v>
       </c>
@@ -3887,7 +3930,7 @@
       <c r="I38" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J38" s="1" t="s">
+      <c r="J38" s="8" t="s">
         <v>506</v>
       </c>
       <c r="K38" s="1" t="s">
@@ -3928,7 +3971,7 @@
       <c r="I39" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J39" s="1" t="s">
+      <c r="J39" s="8" t="s">
         <v>507</v>
       </c>
       <c r="K39" s="1" t="s">
@@ -3941,7 +3984,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>310</v>
       </c>
@@ -3965,7 +4008,7 @@
       <c r="I40" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J40" s="1" t="s">
+      <c r="J40" s="8" t="s">
         <v>510</v>
       </c>
       <c r="K40" s="1" t="s">
@@ -3978,7 +4021,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>241</v>
       </c>
@@ -4006,7 +4049,7 @@
       <c r="I41" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="J41" s="8" t="s">
         <v>509</v>
       </c>
       <c r="K41" s="1" t="s">
@@ -4019,7 +4062,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>251</v>
       </c>
@@ -4047,7 +4090,7 @@
       <c r="I42" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J42" s="1" t="s">
+      <c r="J42" s="8" t="s">
         <v>512</v>
       </c>
       <c r="K42" s="1" t="s">
@@ -4060,7 +4103,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>185</v>
       </c>
@@ -4088,7 +4131,7 @@
       <c r="I43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J43" s="1" t="s">
+      <c r="J43" s="8" t="s">
         <v>513</v>
       </c>
       <c r="K43" s="1" t="s">
@@ -4101,7 +4144,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>177</v>
       </c>
@@ -4125,7 +4168,7 @@
       <c r="I44" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J44" s="1" t="s">
+      <c r="J44" s="8" t="s">
         <v>514</v>
       </c>
       <c r="K44" s="1" t="s">
@@ -4138,7 +4181,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>256</v>
       </c>
@@ -4166,7 +4209,7 @@
       <c r="I45" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J45" s="1" t="s">
+      <c r="J45" s="8" t="s">
         <v>515</v>
       </c>
       <c r="K45" s="1" t="s">
@@ -4179,7 +4222,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>130</v>
       </c>
@@ -4207,7 +4250,7 @@
       <c r="I46" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="J46" s="8" t="s">
         <v>508</v>
       </c>
       <c r="K46" s="1" t="s">
@@ -4220,7 +4263,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>277</v>
       </c>
@@ -4248,7 +4291,7 @@
       <c r="I47" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="J47" s="8" t="s">
         <v>511</v>
       </c>
       <c r="K47" s="1" t="s">
@@ -4261,7 +4304,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>89</v>
       </c>
@@ -4289,7 +4332,7 @@
       <c r="I48" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J48" s="1" t="s">
+      <c r="J48" s="8" t="s">
         <v>543</v>
       </c>
       <c r="K48" s="1" t="s">
@@ -4302,7 +4345,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>56</v>
       </c>
@@ -4330,7 +4373,7 @@
       <c r="I49" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J49" s="1" t="s">
+      <c r="J49" s="8" t="s">
         <v>560</v>
       </c>
       <c r="K49" s="1" t="s">
@@ -4343,7 +4386,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>246</v>
       </c>
@@ -4371,7 +4414,7 @@
       <c r="I50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J50" s="1" t="s">
+      <c r="J50" s="8" t="s">
         <v>470</v>
       </c>
       <c r="K50" s="1" t="s">
@@ -4384,7 +4427,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>32</v>
       </c>
@@ -4412,7 +4455,7 @@
       <c r="I51" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J51" s="3" t="s">
+      <c r="J51" s="9" t="s">
         <v>594</v>
       </c>
       <c r="K51" s="1" t="s">
@@ -4453,7 +4496,7 @@
       <c r="I52" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J52" s="1" t="s">
+      <c r="J52" s="8" t="s">
         <v>604</v>
       </c>
       <c r="K52" s="1" t="s">
@@ -4466,7 +4509,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>212</v>
       </c>
@@ -4494,7 +4537,7 @@
       <c r="I53" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J53" s="1" t="s">
+      <c r="J53" s="8" t="s">
         <v>516</v>
       </c>
       <c r="K53" s="1" t="s">
@@ -4507,7 +4550,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>259</v>
       </c>
@@ -4535,7 +4578,7 @@
       <c r="I54" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J54" s="1" t="s">
+      <c r="J54" s="8" t="s">
         <v>517</v>
       </c>
       <c r="K54" s="1" t="s">
@@ -4548,7 +4591,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>306</v>
       </c>
@@ -4572,7 +4615,7 @@
       <c r="I55" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J55" s="1" t="s">
+      <c r="J55" s="8" t="s">
         <v>518</v>
       </c>
       <c r="K55" s="1" t="s">
@@ -4585,7 +4628,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>323</v>
       </c>
@@ -4609,7 +4652,7 @@
       <c r="I56" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J56" s="1" t="s">
+      <c r="J56" s="8" t="s">
         <v>519</v>
       </c>
       <c r="K56" s="1" t="s">
@@ -4622,7 +4665,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>326</v>
       </c>
@@ -4646,7 +4689,7 @@
       <c r="I57" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J57" s="1" t="s">
+      <c r="J57" s="8" t="s">
         <v>589</v>
       </c>
       <c r="K57" s="1" t="s">
@@ -4659,7 +4702,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>32</v>
       </c>
@@ -4687,7 +4730,7 @@
       <c r="I58" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="J58" s="1" t="s">
+      <c r="J58" s="8" t="s">
         <v>601</v>
       </c>
       <c r="K58" s="1" t="s">
@@ -4700,7 +4743,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>282</v>
       </c>
@@ -4728,7 +4771,7 @@
       <c r="I59" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J59" s="1" t="s">
+      <c r="J59" s="8" t="s">
         <v>540</v>
       </c>
       <c r="K59" s="1" t="s">
@@ -4741,7 +4784,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>272</v>
       </c>
@@ -4769,7 +4812,7 @@
       <c r="I60" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J60" s="1" t="s">
+      <c r="J60" s="8" t="s">
         <v>541</v>
       </c>
       <c r="K60" s="1" t="s">
@@ -4782,7 +4825,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>149</v>
       </c>
@@ -4806,7 +4849,7 @@
       <c r="I61" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J61" s="1" t="s">
+      <c r="J61" s="8" t="s">
         <v>542</v>
       </c>
       <c r="K61" s="1" t="s">
@@ -4819,7 +4862,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>152</v>
       </c>
@@ -4847,7 +4890,7 @@
       <c r="I62" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J62" s="1" t="s">
+      <c r="J62" s="8" t="s">
         <v>544</v>
       </c>
       <c r="K62" s="1" t="s">
@@ -4860,7 +4903,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>221</v>
       </c>
@@ -4888,7 +4931,7 @@
       <c r="I63" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J63" s="1" t="s">
+      <c r="J63" s="8" t="s">
         <v>546</v>
       </c>
       <c r="K63" s="1" t="s">
@@ -4901,7 +4944,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>313</v>
       </c>
@@ -4925,7 +4968,7 @@
       <c r="I64" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J64" s="1" t="s">
+      <c r="J64" s="8" t="s">
         <v>547</v>
       </c>
       <c r="K64" s="1" t="s">
@@ -4938,7 +4981,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>320</v>
       </c>
@@ -4962,7 +5005,7 @@
       <c r="I65" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J65" s="1" t="s">
+      <c r="J65" s="8" t="s">
         <v>548</v>
       </c>
       <c r="K65" s="1" t="s">
@@ -4975,7 +5018,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>317</v>
       </c>
@@ -4999,7 +5042,7 @@
       <c r="I66" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J66" s="1" t="s">
+      <c r="J66" s="8" t="s">
         <v>549</v>
       </c>
       <c r="K66" s="1" t="s">
@@ -5012,7 +5055,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>190</v>
       </c>
@@ -5036,7 +5079,7 @@
       <c r="I67" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J67" s="1" t="s">
+      <c r="J67" s="8" t="s">
         <v>545</v>
       </c>
       <c r="K67" s="1" t="s">
@@ -5049,7 +5092,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>413</v>
       </c>
@@ -5073,7 +5116,7 @@
       <c r="I68" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J68" s="1" t="s">
+      <c r="J68" s="8" t="s">
         <v>550</v>
       </c>
       <c r="K68" s="1" t="s">
@@ -5110,7 +5153,7 @@
       <c r="I69" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J69" s="1" t="s">
+      <c r="J69" s="8" t="s">
         <v>551</v>
       </c>
       <c r="K69" s="1" t="s">
@@ -5123,7 +5166,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>458</v>
       </c>
@@ -5147,7 +5190,7 @@
       <c r="I70" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J70" s="1" t="s">
+      <c r="J70" s="8" t="s">
         <v>552</v>
       </c>
       <c r="K70" s="1" t="s">
@@ -5160,7 +5203,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>156</v>
       </c>
@@ -5184,7 +5227,7 @@
       <c r="I71" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J71" s="1" t="s">
+      <c r="J71" s="8" t="s">
         <v>553</v>
       </c>
       <c r="K71" s="1" t="s">
@@ -5197,7 +5240,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>159</v>
       </c>
@@ -5221,7 +5264,7 @@
       <c r="I72" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J72" s="1" t="s">
+      <c r="J72" s="8" t="s">
         <v>554</v>
       </c>
       <c r="K72" s="1" t="s">
@@ -5234,7 +5277,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>162</v>
       </c>
@@ -5258,7 +5301,7 @@
       <c r="I73" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J73" s="1" t="s">
+      <c r="J73" s="8" t="s">
         <v>555</v>
       </c>
       <c r="K73" s="1" t="s">
@@ -5271,7 +5314,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>216</v>
       </c>
@@ -5299,7 +5342,7 @@
       <c r="I74" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J74" s="1" t="s">
+      <c r="J74" s="8" t="s">
         <v>556</v>
       </c>
       <c r="K74" s="1" t="s">
@@ -5312,7 +5355,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>69</v>
       </c>
@@ -5340,7 +5383,7 @@
       <c r="I75" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J75" s="1" t="s">
+      <c r="J75" s="8" t="s">
         <v>557</v>
       </c>
       <c r="K75" s="1" t="s">
@@ -5353,7 +5396,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>205</v>
       </c>
@@ -5381,7 +5424,7 @@
       <c r="I76" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J76" s="1" t="s">
+      <c r="J76" s="8" t="s">
         <v>558</v>
       </c>
       <c r="K76" s="1" t="s">
@@ -5394,7 +5437,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>135</v>
       </c>
@@ -5422,7 +5465,7 @@
       <c r="I77" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J77" s="1" t="s">
+      <c r="J77" s="8" t="s">
         <v>559</v>
       </c>
       <c r="K77" s="1" t="s">
@@ -5435,7 +5478,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>294</v>
       </c>
@@ -5459,7 +5502,7 @@
       <c r="I78" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J78" s="1" t="s">
+      <c r="J78" s="8" t="s">
         <v>561</v>
       </c>
       <c r="K78" s="1" t="s">
@@ -5472,7 +5515,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>362</v>
       </c>
@@ -5496,7 +5539,7 @@
       <c r="I79" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J79" s="1" t="s">
+      <c r="J79" s="8" t="s">
         <v>562</v>
       </c>
       <c r="K79" s="1" t="s">
@@ -5533,7 +5576,7 @@
       <c r="I80" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J80" s="1" t="s">
+      <c r="J80" s="8" t="s">
         <v>563</v>
       </c>
       <c r="K80" s="1" t="s">
@@ -5546,7 +5589,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>141</v>
       </c>
@@ -5570,7 +5613,7 @@
       <c r="I81" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J81" s="1" t="s">
+      <c r="J81" s="8" t="s">
         <v>564</v>
       </c>
       <c r="K81" s="1" t="s">
@@ -5583,7 +5626,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>164</v>
       </c>
@@ -5607,7 +5650,7 @@
       <c r="I82" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J82" s="1" t="s">
+      <c r="J82" s="8" t="s">
         <v>565</v>
       </c>
       <c r="K82" s="1" t="s">
@@ -5620,7 +5663,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>77</v>
       </c>
@@ -5648,7 +5691,7 @@
       <c r="I83" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J83" s="1" t="s">
+      <c r="J83" s="8" t="s">
         <v>566</v>
       </c>
       <c r="K83" s="1" t="s">
@@ -5689,7 +5732,7 @@
       <c r="I84" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J84" s="1" t="s">
+      <c r="J84" s="8" t="s">
         <v>568</v>
       </c>
       <c r="K84" s="1" t="s">
@@ -5730,7 +5773,7 @@
       <c r="I85" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J85" s="1" t="s">
+      <c r="J85" s="8" t="s">
         <v>569</v>
       </c>
       <c r="K85" s="1" t="s">
@@ -5771,8 +5814,8 @@
       <c r="I86" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J86" s="1" t="s">
-        <v>607</v>
+      <c r="J86" s="8" t="s">
+        <v>646</v>
       </c>
       <c r="K86" s="1" t="s">
         <v>21</v>
@@ -5812,7 +5855,7 @@
       <c r="I87" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J87" s="1" t="s">
+      <c r="J87" s="8" t="s">
         <v>570</v>
       </c>
       <c r="K87" s="1" t="s">
@@ -5853,8 +5896,8 @@
       <c r="I88" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J88" s="3" t="s">
-        <v>606</v>
+      <c r="J88" s="9" t="s">
+        <v>645</v>
       </c>
       <c r="K88" s="1" t="s">
         <v>21</v>
@@ -5894,7 +5937,7 @@
       <c r="I89" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J89" s="1" t="s">
+      <c r="J89" s="8" t="s">
         <v>571</v>
       </c>
       <c r="K89" s="1" t="s">
@@ -5931,8 +5974,8 @@
       <c r="I90" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J90" s="1" t="s">
-        <v>605</v>
+      <c r="J90" s="8" t="s">
+        <v>647</v>
       </c>
       <c r="K90" s="1" t="s">
         <v>21</v>
@@ -5972,7 +6015,7 @@
       <c r="I91" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J91" s="3" t="s">
+      <c r="J91" s="9" t="s">
         <v>597</v>
       </c>
       <c r="K91" s="1" t="s">
@@ -6009,7 +6052,7 @@
       <c r="I92" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J92" s="1" t="s">
+      <c r="J92" s="8" t="s">
         <v>572</v>
       </c>
       <c r="K92" s="1" t="s">
@@ -6046,7 +6089,7 @@
       <c r="I93" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J93" s="1" t="s">
+      <c r="J93" s="8" t="s">
         <v>573</v>
       </c>
       <c r="K93" s="1" t="s">
@@ -6087,7 +6130,7 @@
       <c r="I94" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J94" s="1" t="s">
+      <c r="J94" s="8" t="s">
         <v>574</v>
       </c>
       <c r="K94" s="1" t="s">
@@ -6128,7 +6171,7 @@
       <c r="I95" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J95" s="1" t="s">
+      <c r="J95" s="8" t="s">
         <v>567</v>
       </c>
       <c r="K95" s="1" t="s">
@@ -6169,7 +6212,7 @@
       <c r="I96" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J96" s="1" t="s">
+      <c r="J96" s="8" t="s">
         <v>575</v>
       </c>
       <c r="K96" s="1" t="s">
@@ -6182,7 +6225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>454</v>
       </c>
@@ -6206,7 +6249,7 @@
       <c r="I97" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J97" s="1" t="s">
+      <c r="J97" s="8" t="s">
         <v>576</v>
       </c>
       <c r="K97" s="1" t="s">
@@ -6219,7 +6262,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>200</v>
       </c>
@@ -6247,7 +6290,7 @@
       <c r="I98" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J98" s="1" t="s">
+      <c r="J98" s="8" t="s">
         <v>577</v>
       </c>
       <c r="K98" s="1" t="s">
@@ -6260,7 +6303,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>364</v>
       </c>
@@ -6284,7 +6327,7 @@
       <c r="I99" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J99" s="1" t="s">
+      <c r="J99" s="8" t="s">
         <v>578</v>
       </c>
       <c r="K99" s="1" t="s">
@@ -6297,7 +6340,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>297</v>
       </c>
@@ -6321,7 +6364,7 @@
       <c r="I100" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J100" s="1" t="s">
+      <c r="J100" s="8" t="s">
         <v>579</v>
       </c>
       <c r="K100" s="1" t="s">
@@ -6334,7 +6377,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>378</v>
       </c>
@@ -6358,7 +6401,7 @@
       <c r="I101" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J101" s="1" t="s">
+      <c r="J101" s="8" t="s">
         <v>580</v>
       </c>
       <c r="K101" s="1" t="s">
@@ -6371,7 +6414,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>167</v>
       </c>
@@ -6395,7 +6438,7 @@
       <c r="I102" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J102" s="1" t="s">
+      <c r="J102" s="8" t="s">
         <v>581</v>
       </c>
       <c r="K102" s="1" t="s">
@@ -6408,7 +6451,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>97</v>
       </c>
@@ -6436,7 +6479,7 @@
       <c r="I103" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J103" s="1" t="s">
+      <c r="J103" s="8" t="s">
         <v>582</v>
       </c>
       <c r="K103" s="1" t="s">
@@ -6449,7 +6492,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>127</v>
       </c>
@@ -6477,7 +6520,7 @@
       <c r="I104" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J104" s="1" t="s">
+      <c r="J104" s="8" t="s">
         <v>583</v>
       </c>
       <c r="K104" s="1" t="s">
@@ -6490,7 +6533,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>100</v>
       </c>
@@ -6518,7 +6561,7 @@
       <c r="I105" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J105" s="1" t="s">
+      <c r="J105" s="8" t="s">
         <v>584</v>
       </c>
       <c r="K105" s="1" t="s">
@@ -6559,7 +6602,7 @@
       <c r="I106" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J106" s="1" t="s">
+      <c r="J106" s="8" t="s">
         <v>586</v>
       </c>
       <c r="K106" s="1" t="s">
@@ -6572,7 +6615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>231</v>
       </c>
@@ -6600,7 +6643,7 @@
       <c r="I107" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J107" s="1" t="s">
+      <c r="J107" s="8" t="s">
         <v>585</v>
       </c>
       <c r="K107" s="1" t="s">
@@ -6613,7 +6656,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>195</v>
       </c>
@@ -6637,7 +6680,7 @@
       <c r="I108" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="J108" s="1" t="s">
+      <c r="J108" s="8" t="s">
         <v>587</v>
       </c>
       <c r="K108" s="1" t="s">
@@ -6650,7 +6693,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>353</v>
       </c>
@@ -6674,7 +6717,7 @@
       <c r="I109" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J109" s="1" t="s">
+      <c r="J109" s="8" t="s">
         <v>588</v>
       </c>
       <c r="K109" s="1" t="s">
@@ -6687,7 +6730,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>45</v>
       </c>
@@ -6715,7 +6758,7 @@
       <c r="I110" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J110" s="1" t="s">
+      <c r="J110" s="8" t="s">
         <v>539</v>
       </c>
       <c r="K110" s="1" t="s">
@@ -6728,7 +6771,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>173</v>
       </c>
@@ -6756,7 +6799,7 @@
       <c r="I111" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J111" s="1" t="s">
+      <c r="J111" s="8" t="s">
         <v>538</v>
       </c>
       <c r="K111" s="1" t="s">
@@ -6769,7 +6812,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>124</v>
       </c>
@@ -6797,7 +6840,7 @@
       <c r="I112" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J112" s="1" t="s">
+      <c r="J112" s="8" t="s">
         <v>537</v>
       </c>
       <c r="K112" s="1" t="s">
@@ -6810,7 +6853,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>53</v>
       </c>
@@ -6838,7 +6881,7 @@
       <c r="I113" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J113" s="1" t="s">
+      <c r="J113" s="8" t="s">
         <v>536</v>
       </c>
       <c r="K113" s="1" t="s">
@@ -6875,7 +6918,7 @@
       <c r="I114" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J114" s="1" t="s">
+      <c r="J114" s="8" t="s">
         <v>535</v>
       </c>
       <c r="K114" s="1" t="s">
@@ -6888,7 +6931,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>12</v>
       </c>
@@ -6916,7 +6959,7 @@
       <c r="I115" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J115" s="1" t="s">
+      <c r="J115" s="8" t="s">
         <v>534</v>
       </c>
       <c r="K115" s="1" t="s">
@@ -6929,7 +6972,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>181</v>
       </c>
@@ -6957,7 +7000,7 @@
       <c r="I116" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J116" s="1" t="s">
+      <c r="J116" s="8" t="s">
         <v>533</v>
       </c>
       <c r="K116" s="1" t="s">
@@ -6970,7 +7013,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>359</v>
       </c>
@@ -6994,7 +7037,7 @@
       <c r="I117" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J117" s="1" t="s">
+      <c r="J117" s="8" t="s">
         <v>532</v>
       </c>
       <c r="K117" s="1" t="s">
@@ -7007,7 +7050,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>170</v>
       </c>
@@ -7031,7 +7074,7 @@
       <c r="I118" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J118" s="1" t="s">
+      <c r="J118" s="8" t="s">
         <v>531</v>
       </c>
       <c r="K118" s="1" t="s">
@@ -7044,7 +7087,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>103</v>
       </c>
@@ -7072,7 +7115,7 @@
       <c r="I119" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J119" s="1" t="s">
+      <c r="J119" s="8" t="s">
         <v>530</v>
       </c>
       <c r="K119" s="1" t="s">
@@ -7085,7 +7128,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>288</v>
       </c>
@@ -7109,7 +7152,7 @@
       <c r="I120" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J120" s="1" t="s">
+      <c r="J120" s="8" t="s">
         <v>529</v>
       </c>
       <c r="K120" s="1" t="s">
@@ -7122,7 +7165,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>81</v>
       </c>
@@ -7150,7 +7193,7 @@
       <c r="I121" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J121" s="1" t="s">
+      <c r="J121" s="8" t="s">
         <v>527</v>
       </c>
       <c r="K121" s="1" t="s">
@@ -7163,7 +7206,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>86</v>
       </c>
@@ -7191,7 +7234,7 @@
       <c r="I122" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J122" s="1" t="s">
+      <c r="J122" s="8" t="s">
         <v>526</v>
       </c>
       <c r="K122" s="4" t="s">
@@ -7204,7 +7247,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="123" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:13" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>92</v>
       </c>
@@ -7232,7 +7275,7 @@
       <c r="I123" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J123" s="1" t="s">
+      <c r="J123" s="8" t="s">
         <v>525</v>
       </c>
       <c r="K123" s="1" t="s">
@@ -7245,7 +7288,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
         <v>74</v>
       </c>
@@ -7273,7 +7316,7 @@
       <c r="I124" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J124" s="5" t="s">
+      <c r="J124" s="10" t="s">
         <v>528</v>
       </c>
       <c r="K124" s="5" t="s">
@@ -7286,7 +7329,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>106</v>
       </c>
@@ -7314,7 +7357,7 @@
       <c r="I125" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J125" s="1" t="s">
+      <c r="J125" s="8" t="s">
         <v>524</v>
       </c>
       <c r="K125" s="1" t="s">
@@ -7327,7 +7370,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>109</v>
       </c>
@@ -7355,7 +7398,7 @@
       <c r="I126" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J126" s="1" t="s">
+      <c r="J126" s="8" t="s">
         <v>523</v>
       </c>
       <c r="K126" s="1" t="s">
@@ -7368,7 +7411,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>112</v>
       </c>
@@ -7396,7 +7439,7 @@
       <c r="I127" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J127" s="1" t="s">
+      <c r="J127" s="8" t="s">
         <v>522</v>
       </c>
       <c r="K127" s="1" t="s">
@@ -7409,7 +7452,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>303</v>
       </c>
@@ -7433,7 +7476,7 @@
       <c r="I128" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J128" s="1" t="s">
+      <c r="J128" s="8" t="s">
         <v>521</v>
       </c>
       <c r="K128" s="1" t="s">
@@ -7446,7 +7489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>32</v>
       </c>
@@ -7474,7 +7517,7 @@
       <c r="I129" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J129" s="1" t="s">
+      <c r="J129" s="8" t="s">
         <v>590</v>
       </c>
       <c r="K129" s="1" t="s">
@@ -7487,7 +7530,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>32</v>
       </c>
@@ -7515,7 +7558,7 @@
       <c r="I130" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J130" s="1" t="s">
+      <c r="J130" s="8" t="s">
         <v>520</v>
       </c>
       <c r="K130" s="1" t="s">
@@ -7528,36 +7571,36 @@
         <v>23</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>608</v>
+        <v>34</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>15</v>
+        <v>605</v>
       </c>
       <c r="E131" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>17</v>
+        <v>606</v>
       </c>
       <c r="G131" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H131" s="1" t="s">
-        <v>19</v>
+        <v>607</v>
       </c>
       <c r="I131" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J131" s="1" t="s">
-        <v>621</v>
+      <c r="J131" s="8" t="s">
+        <v>637</v>
       </c>
       <c r="K131" s="1" t="s">
         <v>21</v>
@@ -7566,39 +7609,39 @@
         <v>22</v>
       </c>
       <c r="M131" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C132" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D132" s="1" t="s">
         <v>609</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="E132" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>17</v>
+        <v>610</v>
       </c>
       <c r="G132" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H132" s="1" t="s">
-        <v>19</v>
+        <v>611</v>
       </c>
       <c r="I132" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J132" s="1" t="s">
-        <v>622</v>
+      <c r="J132" s="8" t="s">
+        <v>638</v>
       </c>
       <c r="K132" s="1" t="s">
         <v>21</v>
@@ -7607,39 +7650,39 @@
         <v>22</v>
       </c>
       <c r="M132" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="133" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B133" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>610</v>
+        <v>34</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>15</v>
+        <v>613</v>
       </c>
       <c r="E133" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>17</v>
+        <v>614</v>
       </c>
       <c r="G133" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H133" s="1" t="s">
-        <v>19</v>
+        <v>615</v>
       </c>
       <c r="I133" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J133" s="1" t="s">
-        <v>623</v>
+      <c r="J133" s="8" t="s">
+        <v>639</v>
       </c>
       <c r="K133" s="1" t="s">
         <v>21</v>
@@ -7648,39 +7691,39 @@
         <v>22</v>
       </c>
       <c r="M133" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="134" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>611</v>
+        <v>34</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>15</v>
+        <v>617</v>
       </c>
       <c r="E134" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>17</v>
+        <v>618</v>
       </c>
       <c r="G134" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H134" s="1" t="s">
-        <v>19</v>
+        <v>619</v>
       </c>
       <c r="I134" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J134" s="1" t="s">
-        <v>612</v>
+      <c r="J134" s="8" t="s">
+        <v>640</v>
       </c>
       <c r="K134" s="1" t="s">
         <v>21</v>
@@ -7689,80 +7732,80 @@
         <v>22</v>
       </c>
       <c r="M134" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="135" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>613</v>
+        <v>34</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>15</v>
+        <v>621</v>
       </c>
       <c r="E135" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>17</v>
+        <v>622</v>
       </c>
       <c r="G135" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>19</v>
+        <v>623</v>
       </c>
       <c r="I135" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J135" s="1" t="s">
+      <c r="J135" s="8" t="s">
+        <v>641</v>
+      </c>
+      <c r="K135" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L135" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M135" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="K135" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L135" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M135" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="136" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>614</v>
+        <v>34</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>15</v>
+        <v>625</v>
       </c>
       <c r="E136" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>17</v>
+        <v>626</v>
       </c>
       <c r="G136" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H136" s="1" t="s">
-        <v>19</v>
+        <v>627</v>
       </c>
       <c r="I136" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J136" s="1" t="s">
-        <v>625</v>
+      <c r="J136" s="8" t="s">
+        <v>642</v>
       </c>
       <c r="K136" s="1" t="s">
         <v>21</v>
@@ -7771,39 +7814,39 @@
         <v>22</v>
       </c>
       <c r="M136" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="137" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>615</v>
+        <v>34</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>15</v>
+        <v>629</v>
       </c>
       <c r="E137" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F137" s="1" t="s">
-        <v>17</v>
+        <v>630</v>
       </c>
       <c r="G137" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>19</v>
+        <v>631</v>
       </c>
       <c r="I137" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J137" s="1" t="s">
-        <v>626</v>
+      <c r="J137" s="8" t="s">
+        <v>643</v>
       </c>
       <c r="K137" s="1" t="s">
         <v>21</v>
@@ -7812,39 +7855,39 @@
         <v>22</v>
       </c>
       <c r="M137" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="138" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>616</v>
+        <v>34</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>15</v>
+        <v>633</v>
       </c>
       <c r="E138" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F138" s="1" t="s">
-        <v>17</v>
+        <v>634</v>
       </c>
       <c r="G138" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>19</v>
+        <v>635</v>
       </c>
       <c r="I138" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J138" s="1" t="s">
-        <v>627</v>
+      <c r="J138" s="8" t="s">
+        <v>644</v>
       </c>
       <c r="K138" s="1" t="s">
         <v>21</v>
@@ -7853,175 +7896,16 @@
         <v>22</v>
       </c>
       <c r="M138" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A139" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B139" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C139" s="7" t="s">
-        <v>617</v>
-      </c>
-      <c r="D139" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E139" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F139" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G139" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H139" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I139" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J139" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="K139" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L139" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M139" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A140" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B140" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>618</v>
-      </c>
-      <c r="D140" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F140" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G140" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H140" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I140" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J140" s="1" t="s">
-        <v>628</v>
-      </c>
-      <c r="K140" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L140" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M140" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A141" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B141" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C141" s="1" t="s">
-        <v>619</v>
-      </c>
-      <c r="D141" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E141" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F141" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G141" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H141" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I141" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J141" s="1" t="s">
-        <v>630</v>
-      </c>
-      <c r="K141" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L141" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M141" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A142" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B142" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C142" s="1" t="s">
-        <v>620</v>
-      </c>
-      <c r="D142" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E142" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F142" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G142" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H142" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I142" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J142" s="1" t="s">
-        <v>629</v>
-      </c>
-      <c r="K142" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L142" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M142" s="1" t="s">
-        <v>23</v>
+        <v>636</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M142" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:M138" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="GRD00001"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M130">
       <sortCondition ref="J1:J130"/>
     </sortState>
@@ -8029,20 +7913,15 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M116">
     <sortCondition ref="C1:C116"/>
   </sortState>
-  <conditionalFormatting sqref="C140:C142 C131:C138">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="C1:C126">
+    <cfRule type="duplicateValues" dxfId="2" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C143:C1048576 C1:C126">
-    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+  <conditionalFormatting sqref="C127:C138">
+    <cfRule type="duplicateValues" dxfId="1" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J131:J142">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J143:J1048576 J1:J130">
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C127:C130">
-    <cfRule type="duplicateValues" dxfId="0" priority="39"/>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add RMT automation framework with secure runtime configuration
Adds allocation and configuration automation, reporting, CI/CD, MCP tooling, and runtime-only credential handling.
</commit_message>
<xml_diff>
--- a/src/test/TestData/Designation Master.xlsx
+++ b/src/test/TestData/Designation Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Piyush.Wadhwa\IdeaProjects\Automation\RMT\src\test\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2052208A-D4FC-4C55-BD7A-CCF56FBE8E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CAB125-E6E2-412E-A7A4-185330CDB570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Designation Master" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Designation Master'!$A$1:$M$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Designation Master'!$A$1:$M$138</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1726" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1674" uniqueCount="648">
   <si>
     <t>DESGN_ID</t>
   </si>
@@ -1853,82 +1853,133 @@
     <t>//li[text()='Clients &amp; Markets Leader - Advisory Services']</t>
   </si>
   <si>
-    <t>//li[text()='Partner and Leader – Private Client Services']</t>
-  </si>
-  <si>
-    <t>//li[text()='Partner &amp; COO']</t>
-  </si>
-  <si>
-    <t>//li[text()='Partner – National Management']</t>
-  </si>
-  <si>
-    <t>ASSISTANT MANAGER WINGS</t>
-  </si>
-  <si>
-    <t>ASSOCIATE DIRECTOR WINGS</t>
-  </si>
-  <si>
-    <t>CONSULTANT WINGS</t>
-  </si>
-  <si>
-    <t>CSS4 WINGS</t>
-  </si>
-  <si>
-    <t>//li[text()='CSS4 WINGS']</t>
-  </si>
-  <si>
-    <t>DIRECTOR WINGS</t>
-  </si>
-  <si>
-    <t>DIRECTOR – IKCC</t>
-  </si>
-  <si>
-    <t>EXECUTIVE DIRECTOR WINGS</t>
-  </si>
-  <si>
-    <t>MANAGER WINGS</t>
-  </si>
-  <si>
-    <t>PARTNER - CLIENTS &amp; MARKETS</t>
-  </si>
-  <si>
-    <t>PARTNER-WINGS</t>
-  </si>
-  <si>
-    <t>RMS TESTING</t>
-  </si>
-  <si>
-    <t>TRAINEE WINGS</t>
-  </si>
-  <si>
-    <t>//li[text()='Assistant Manager WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Associate Director WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Consultant WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Director WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Director – IKCC']</t>
-  </si>
-  <si>
-    <t>//li[text()='Executive Director WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Manager WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Partner-WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='Trainee WINGS']</t>
-  </si>
-  <si>
-    <t>//li[text()='RMS Testing']</t>
+    <t>US000013</t>
+  </si>
+  <si>
+    <t>US000002</t>
+  </si>
+  <si>
+    <t>04-OCT-11</t>
+  </si>
+  <si>
+    <t>08-NOV-25</t>
+  </si>
+  <si>
+    <t>US000014</t>
+  </si>
+  <si>
+    <t>US000003</t>
+  </si>
+  <si>
+    <t>04-OCT-12</t>
+  </si>
+  <si>
+    <t>08-NOV-26</t>
+  </si>
+  <si>
+    <t>US000015</t>
+  </si>
+  <si>
+    <t>US000004</t>
+  </si>
+  <si>
+    <t>04-OCT-13</t>
+  </si>
+  <si>
+    <t>08-NOV-27</t>
+  </si>
+  <si>
+    <t>US000016</t>
+  </si>
+  <si>
+    <t>US000005</t>
+  </si>
+  <si>
+    <t>04-OCT-14</t>
+  </si>
+  <si>
+    <t>08-NOV-28</t>
+  </si>
+  <si>
+    <t>US000017</t>
+  </si>
+  <si>
+    <t>US000006</t>
+  </si>
+  <si>
+    <t>04-OCT-15</t>
+  </si>
+  <si>
+    <t>08-NOV-29</t>
+  </si>
+  <si>
+    <t>US000018</t>
+  </si>
+  <si>
+    <t>US000007</t>
+  </si>
+  <si>
+    <t>04-OCT-16</t>
+  </si>
+  <si>
+    <t>08-NOV-30</t>
+  </si>
+  <si>
+    <t>US000019</t>
+  </si>
+  <si>
+    <t>US000008</t>
+  </si>
+  <si>
+    <t>04-OCT-17</t>
+  </si>
+  <si>
+    <t>08-NOV-31</t>
+  </si>
+  <si>
+    <t>US000020</t>
+  </si>
+  <si>
+    <t>US000009</t>
+  </si>
+  <si>
+    <t>04-OCT-18</t>
+  </si>
+  <si>
+    <t>08-NOV-32</t>
+  </si>
+  <si>
+    <t>//li[text()='Associate Consultant']</t>
+  </si>
+  <si>
+    <t>//li[text()='Change Management Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Chief Information Officer']</t>
+  </si>
+  <si>
+    <t>//li[text()='Client Experience Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner,CPCO']</t>
+  </si>
+  <si>
+    <t>//li[text()='Strategic Sourcing Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Transformation &amp; Innovation Leader']</t>
+  </si>
+  <si>
+    <t>//li[text()='Travel Incharge - Office of the CEO']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner, COO']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner - National Managementment']</t>
+  </si>
+  <si>
+    <t>//li[text()='Partner and Leader - Private Client Services']</t>
   </si>
 </sst>
 </file>
@@ -1952,7 +2003,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2031,7 +2082,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2049,34 +2100,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2417,10 +2460,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M142"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.77734375" customWidth="1"/>
@@ -2432,7 +2475,7 @@
     <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16.88671875" customWidth="1"/>
-    <col min="10" max="10" width="68.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="68.77734375" style="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -2466,7 +2509,7 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="7" t="s">
         <v>469</v>
       </c>
       <c r="K1" s="2" t="s">
@@ -2479,7 +2522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -2507,7 +2550,7 @@
       <c r="I2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="8" t="s">
         <v>593</v>
       </c>
       <c r="K2" s="1" t="s">
@@ -2544,7 +2587,7 @@
       <c r="I3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="8" t="s">
         <v>471</v>
       </c>
       <c r="K3" s="1" t="s">
@@ -2557,7 +2600,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
@@ -2585,7 +2628,7 @@
       <c r="I4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="8" t="s">
         <v>472</v>
       </c>
       <c r="K4" s="1" t="s">
@@ -2598,7 +2641,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
@@ -2626,7 +2669,7 @@
       <c r="I5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="8" t="s">
         <v>473</v>
       </c>
       <c r="K5" s="1" t="s">
@@ -2663,7 +2706,7 @@
       <c r="I6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="8" t="s">
         <v>476</v>
       </c>
       <c r="K6" s="1" t="s">
@@ -2704,7 +2747,7 @@
       <c r="I7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="8" t="s">
         <v>475</v>
       </c>
       <c r="K7" s="1" t="s">
@@ -2717,7 +2760,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>350</v>
       </c>
@@ -2741,7 +2784,7 @@
       <c r="I8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="8" t="s">
         <v>477</v>
       </c>
       <c r="K8" s="1" t="s">
@@ -2754,7 +2797,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
@@ -2782,7 +2825,7 @@
       <c r="I9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="8" t="s">
         <v>478</v>
       </c>
       <c r="K9" s="1" t="s">
@@ -2795,7 +2838,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>118</v>
       </c>
@@ -2823,7 +2866,7 @@
       <c r="I10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="8" t="s">
         <v>479</v>
       </c>
       <c r="K10" s="1" t="s">
@@ -2836,7 +2879,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>121</v>
       </c>
@@ -2864,7 +2907,7 @@
       <c r="I11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="8" t="s">
         <v>480</v>
       </c>
       <c r="K11" s="1" t="s">
@@ -2877,7 +2920,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>64</v>
       </c>
@@ -2905,7 +2948,7 @@
       <c r="I12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="8" t="s">
         <v>474</v>
       </c>
       <c r="K12" s="1" t="s">
@@ -2918,7 +2961,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>408</v>
       </c>
@@ -2946,7 +2989,7 @@
       <c r="I13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="8" t="s">
         <v>481</v>
       </c>
       <c r="K13" s="1" t="s">
@@ -2987,7 +3030,7 @@
       <c r="I14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="8" t="s">
         <v>482</v>
       </c>
       <c r="K14" s="1" t="s">
@@ -3000,7 +3043,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>115</v>
       </c>
@@ -3028,7 +3071,7 @@
       <c r="I15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="J15" s="8" t="s">
         <v>483</v>
       </c>
       <c r="K15" s="1" t="s">
@@ -3041,7 +3084,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>329</v>
       </c>
@@ -3065,7 +3108,7 @@
       <c r="I16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="J16" s="8" t="s">
         <v>484</v>
       </c>
       <c r="K16" s="1" t="s">
@@ -3078,7 +3121,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>209</v>
       </c>
@@ -3106,7 +3149,7 @@
       <c r="I17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="8" t="s">
         <v>485</v>
       </c>
       <c r="K17" s="1" t="s">
@@ -3143,7 +3186,7 @@
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="8" t="s">
         <v>486</v>
       </c>
       <c r="K18" s="1" t="s">
@@ -3180,7 +3223,7 @@
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="J19" s="8" t="s">
         <v>488</v>
       </c>
       <c r="K19" s="1" t="s">
@@ -3193,7 +3236,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>284</v>
       </c>
@@ -3217,7 +3260,7 @@
       <c r="I20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="1" t="s">
+      <c r="J20" s="8" t="s">
         <v>489</v>
       </c>
       <c r="K20" s="1" t="s">
@@ -3230,7 +3273,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>381</v>
       </c>
@@ -3254,7 +3297,7 @@
       <c r="I21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="J21" s="8" t="s">
         <v>491</v>
       </c>
       <c r="K21" s="1" t="s">
@@ -3267,7 +3310,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>375</v>
       </c>
@@ -3291,7 +3334,7 @@
       <c r="I22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="J22" s="8" t="s">
         <v>487</v>
       </c>
       <c r="K22" s="1" t="s">
@@ -3328,7 +3371,7 @@
       <c r="I23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="J23" s="8" t="s">
         <v>490</v>
       </c>
       <c r="K23" s="1" t="s">
@@ -3341,7 +3384,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>392</v>
       </c>
@@ -3365,7 +3408,7 @@
       <c r="I24" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="J24" s="8" t="s">
         <v>493</v>
       </c>
       <c r="K24" s="1" t="s">
@@ -3402,7 +3445,7 @@
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J25" s="1" t="s">
+      <c r="J25" s="8" t="s">
         <v>494</v>
       </c>
       <c r="K25" s="1" t="s">
@@ -3415,7 +3458,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>396</v>
       </c>
@@ -3439,7 +3482,7 @@
       <c r="I26" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="J26" s="8" t="s">
         <v>492</v>
       </c>
       <c r="K26" s="1" t="s">
@@ -3452,7 +3495,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>49</v>
       </c>
@@ -3480,7 +3523,7 @@
       <c r="I27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J27" s="1" t="s">
+      <c r="J27" s="8" t="s">
         <v>495</v>
       </c>
       <c r="K27" s="1" t="s">
@@ -3493,7 +3536,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>146</v>
       </c>
@@ -3517,7 +3560,7 @@
       <c r="I28" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J28" s="1" t="s">
+      <c r="J28" s="8" t="s">
         <v>496</v>
       </c>
       <c r="K28" s="1" t="s">
@@ -3530,7 +3573,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>366</v>
       </c>
@@ -3554,7 +3597,7 @@
       <c r="I29" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="J29" s="8" t="s">
         <v>497</v>
       </c>
       <c r="K29" s="1" t="s">
@@ -3567,7 +3610,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>419</v>
       </c>
@@ -3591,7 +3634,7 @@
       <c r="I30" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="J30" s="8" t="s">
         <v>498</v>
       </c>
       <c r="K30" s="1" t="s">
@@ -3604,7 +3647,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>356</v>
       </c>
@@ -3628,7 +3671,7 @@
       <c r="I31" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="J31" s="8" t="s">
         <v>499</v>
       </c>
       <c r="K31" s="1" t="s">
@@ -3641,7 +3684,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>347</v>
       </c>
@@ -3665,7 +3708,7 @@
       <c r="I32" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="J32" s="8" t="s">
         <v>500</v>
       </c>
       <c r="K32" s="1" t="s">
@@ -3678,7 +3721,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>369</v>
       </c>
@@ -3702,7 +3745,7 @@
       <c r="I33" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="J33" s="8" t="s">
         <v>502</v>
       </c>
       <c r="K33" s="1" t="s">
@@ -3715,7 +3758,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>300</v>
       </c>
@@ -3739,7 +3782,7 @@
       <c r="I34" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="J34" s="8" t="s">
         <v>501</v>
       </c>
       <c r="K34" s="1" t="s">
@@ -3752,7 +3795,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>343</v>
       </c>
@@ -3776,7 +3819,7 @@
       <c r="I35" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="J35" s="8" t="s">
         <v>503</v>
       </c>
       <c r="K35" s="1" t="s">
@@ -3789,7 +3832,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>416</v>
       </c>
@@ -3813,7 +3856,7 @@
       <c r="I36" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="J36" s="8" t="s">
         <v>504</v>
       </c>
       <c r="K36" s="1" t="s">
@@ -3826,7 +3869,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>291</v>
       </c>
@@ -3850,7 +3893,7 @@
       <c r="I37" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="J37" s="8" t="s">
         <v>505</v>
       </c>
       <c r="K37" s="1" t="s">
@@ -3863,7 +3906,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>372</v>
       </c>
@@ -3887,7 +3930,7 @@
       <c r="I38" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J38" s="1" t="s">
+      <c r="J38" s="8" t="s">
         <v>506</v>
       </c>
       <c r="K38" s="1" t="s">
@@ -3928,7 +3971,7 @@
       <c r="I39" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J39" s="1" t="s">
+      <c r="J39" s="8" t="s">
         <v>507</v>
       </c>
       <c r="K39" s="1" t="s">
@@ -3941,7 +3984,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>310</v>
       </c>
@@ -3965,7 +4008,7 @@
       <c r="I40" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J40" s="1" t="s">
+      <c r="J40" s="8" t="s">
         <v>510</v>
       </c>
       <c r="K40" s="1" t="s">
@@ -3978,7 +4021,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>241</v>
       </c>
@@ -4006,7 +4049,7 @@
       <c r="I41" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="J41" s="8" t="s">
         <v>509</v>
       </c>
       <c r="K41" s="1" t="s">
@@ -4019,7 +4062,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>251</v>
       </c>
@@ -4047,7 +4090,7 @@
       <c r="I42" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J42" s="1" t="s">
+      <c r="J42" s="8" t="s">
         <v>512</v>
       </c>
       <c r="K42" s="1" t="s">
@@ -4060,7 +4103,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>185</v>
       </c>
@@ -4088,7 +4131,7 @@
       <c r="I43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J43" s="1" t="s">
+      <c r="J43" s="8" t="s">
         <v>513</v>
       </c>
       <c r="K43" s="1" t="s">
@@ -4101,7 +4144,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>177</v>
       </c>
@@ -4125,7 +4168,7 @@
       <c r="I44" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J44" s="1" t="s">
+      <c r="J44" s="8" t="s">
         <v>514</v>
       </c>
       <c r="K44" s="1" t="s">
@@ -4138,7 +4181,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>256</v>
       </c>
@@ -4166,7 +4209,7 @@
       <c r="I45" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J45" s="1" t="s">
+      <c r="J45" s="8" t="s">
         <v>515</v>
       </c>
       <c r="K45" s="1" t="s">
@@ -4179,7 +4222,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>130</v>
       </c>
@@ -4207,7 +4250,7 @@
       <c r="I46" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="J46" s="8" t="s">
         <v>508</v>
       </c>
       <c r="K46" s="1" t="s">
@@ -4220,7 +4263,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>277</v>
       </c>
@@ -4248,7 +4291,7 @@
       <c r="I47" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="J47" s="8" t="s">
         <v>511</v>
       </c>
       <c r="K47" s="1" t="s">
@@ -4261,7 +4304,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>89</v>
       </c>
@@ -4289,7 +4332,7 @@
       <c r="I48" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J48" s="1" t="s">
+      <c r="J48" s="8" t="s">
         <v>543</v>
       </c>
       <c r="K48" s="1" t="s">
@@ -4302,7 +4345,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>56</v>
       </c>
@@ -4330,7 +4373,7 @@
       <c r="I49" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J49" s="1" t="s">
+      <c r="J49" s="8" t="s">
         <v>560</v>
       </c>
       <c r="K49" s="1" t="s">
@@ -4343,7 +4386,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>246</v>
       </c>
@@ -4371,7 +4414,7 @@
       <c r="I50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J50" s="1" t="s">
+      <c r="J50" s="8" t="s">
         <v>470</v>
       </c>
       <c r="K50" s="1" t="s">
@@ -4384,7 +4427,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>32</v>
       </c>
@@ -4412,7 +4455,7 @@
       <c r="I51" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J51" s="3" t="s">
+      <c r="J51" s="9" t="s">
         <v>594</v>
       </c>
       <c r="K51" s="1" t="s">
@@ -4453,7 +4496,7 @@
       <c r="I52" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J52" s="1" t="s">
+      <c r="J52" s="8" t="s">
         <v>604</v>
       </c>
       <c r="K52" s="1" t="s">
@@ -4466,7 +4509,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>212</v>
       </c>
@@ -4494,7 +4537,7 @@
       <c r="I53" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J53" s="1" t="s">
+      <c r="J53" s="8" t="s">
         <v>516</v>
       </c>
       <c r="K53" s="1" t="s">
@@ -4507,7 +4550,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>259</v>
       </c>
@@ -4535,7 +4578,7 @@
       <c r="I54" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J54" s="1" t="s">
+      <c r="J54" s="8" t="s">
         <v>517</v>
       </c>
       <c r="K54" s="1" t="s">
@@ -4548,7 +4591,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>306</v>
       </c>
@@ -4572,7 +4615,7 @@
       <c r="I55" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J55" s="1" t="s">
+      <c r="J55" s="8" t="s">
         <v>518</v>
       </c>
       <c r="K55" s="1" t="s">
@@ -4585,7 +4628,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>323</v>
       </c>
@@ -4609,7 +4652,7 @@
       <c r="I56" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J56" s="1" t="s">
+      <c r="J56" s="8" t="s">
         <v>519</v>
       </c>
       <c r="K56" s="1" t="s">
@@ -4622,7 +4665,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>326</v>
       </c>
@@ -4646,7 +4689,7 @@
       <c r="I57" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J57" s="1" t="s">
+      <c r="J57" s="8" t="s">
         <v>589</v>
       </c>
       <c r="K57" s="1" t="s">
@@ -4659,7 +4702,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>32</v>
       </c>
@@ -4687,7 +4730,7 @@
       <c r="I58" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="J58" s="1" t="s">
+      <c r="J58" s="8" t="s">
         <v>601</v>
       </c>
       <c r="K58" s="1" t="s">
@@ -4700,7 +4743,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>282</v>
       </c>
@@ -4728,7 +4771,7 @@
       <c r="I59" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J59" s="1" t="s">
+      <c r="J59" s="8" t="s">
         <v>540</v>
       </c>
       <c r="K59" s="1" t="s">
@@ -4741,7 +4784,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>272</v>
       </c>
@@ -4769,7 +4812,7 @@
       <c r="I60" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J60" s="1" t="s">
+      <c r="J60" s="8" t="s">
         <v>541</v>
       </c>
       <c r="K60" s="1" t="s">
@@ -4782,7 +4825,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>149</v>
       </c>
@@ -4806,7 +4849,7 @@
       <c r="I61" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J61" s="1" t="s">
+      <c r="J61" s="8" t="s">
         <v>542</v>
       </c>
       <c r="K61" s="1" t="s">
@@ -4819,7 +4862,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>152</v>
       </c>
@@ -4847,7 +4890,7 @@
       <c r="I62" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J62" s="1" t="s">
+      <c r="J62" s="8" t="s">
         <v>544</v>
       </c>
       <c r="K62" s="1" t="s">
@@ -4860,7 +4903,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>221</v>
       </c>
@@ -4888,7 +4931,7 @@
       <c r="I63" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J63" s="1" t="s">
+      <c r="J63" s="8" t="s">
         <v>546</v>
       </c>
       <c r="K63" s="1" t="s">
@@ -4901,7 +4944,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>313</v>
       </c>
@@ -4925,7 +4968,7 @@
       <c r="I64" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J64" s="1" t="s">
+      <c r="J64" s="8" t="s">
         <v>547</v>
       </c>
       <c r="K64" s="1" t="s">
@@ -4938,7 +4981,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>320</v>
       </c>
@@ -4962,7 +5005,7 @@
       <c r="I65" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J65" s="1" t="s">
+      <c r="J65" s="8" t="s">
         <v>548</v>
       </c>
       <c r="K65" s="1" t="s">
@@ -4975,7 +5018,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>317</v>
       </c>
@@ -4999,7 +5042,7 @@
       <c r="I66" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J66" s="1" t="s">
+      <c r="J66" s="8" t="s">
         <v>549</v>
       </c>
       <c r="K66" s="1" t="s">
@@ -5012,7 +5055,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>190</v>
       </c>
@@ -5036,7 +5079,7 @@
       <c r="I67" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J67" s="1" t="s">
+      <c r="J67" s="8" t="s">
         <v>545</v>
       </c>
       <c r="K67" s="1" t="s">
@@ -5049,7 +5092,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>413</v>
       </c>
@@ -5073,7 +5116,7 @@
       <c r="I68" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J68" s="1" t="s">
+      <c r="J68" s="8" t="s">
         <v>550</v>
       </c>
       <c r="K68" s="1" t="s">
@@ -5110,7 +5153,7 @@
       <c r="I69" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J69" s="1" t="s">
+      <c r="J69" s="8" t="s">
         <v>551</v>
       </c>
       <c r="K69" s="1" t="s">
@@ -5123,7 +5166,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>458</v>
       </c>
@@ -5147,7 +5190,7 @@
       <c r="I70" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J70" s="1" t="s">
+      <c r="J70" s="8" t="s">
         <v>552</v>
       </c>
       <c r="K70" s="1" t="s">
@@ -5160,7 +5203,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>156</v>
       </c>
@@ -5184,7 +5227,7 @@
       <c r="I71" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J71" s="1" t="s">
+      <c r="J71" s="8" t="s">
         <v>553</v>
       </c>
       <c r="K71" s="1" t="s">
@@ -5197,7 +5240,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>159</v>
       </c>
@@ -5221,7 +5264,7 @@
       <c r="I72" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J72" s="1" t="s">
+      <c r="J72" s="8" t="s">
         <v>554</v>
       </c>
       <c r="K72" s="1" t="s">
@@ -5234,7 +5277,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>162</v>
       </c>
@@ -5258,7 +5301,7 @@
       <c r="I73" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J73" s="1" t="s">
+      <c r="J73" s="8" t="s">
         <v>555</v>
       </c>
       <c r="K73" s="1" t="s">
@@ -5271,7 +5314,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>216</v>
       </c>
@@ -5299,7 +5342,7 @@
       <c r="I74" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J74" s="1" t="s">
+      <c r="J74" s="8" t="s">
         <v>556</v>
       </c>
       <c r="K74" s="1" t="s">
@@ -5312,7 +5355,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>69</v>
       </c>
@@ -5340,7 +5383,7 @@
       <c r="I75" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J75" s="1" t="s">
+      <c r="J75" s="8" t="s">
         <v>557</v>
       </c>
       <c r="K75" s="1" t="s">
@@ -5353,7 +5396,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>205</v>
       </c>
@@ -5381,7 +5424,7 @@
       <c r="I76" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J76" s="1" t="s">
+      <c r="J76" s="8" t="s">
         <v>558</v>
       </c>
       <c r="K76" s="1" t="s">
@@ -5394,7 +5437,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>135</v>
       </c>
@@ -5422,7 +5465,7 @@
       <c r="I77" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J77" s="1" t="s">
+      <c r="J77" s="8" t="s">
         <v>559</v>
       </c>
       <c r="K77" s="1" t="s">
@@ -5435,7 +5478,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>294</v>
       </c>
@@ -5459,7 +5502,7 @@
       <c r="I78" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J78" s="1" t="s">
+      <c r="J78" s="8" t="s">
         <v>561</v>
       </c>
       <c r="K78" s="1" t="s">
@@ -5472,7 +5515,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>362</v>
       </c>
@@ -5496,7 +5539,7 @@
       <c r="I79" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J79" s="1" t="s">
+      <c r="J79" s="8" t="s">
         <v>562</v>
       </c>
       <c r="K79" s="1" t="s">
@@ -5533,7 +5576,7 @@
       <c r="I80" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J80" s="1" t="s">
+      <c r="J80" s="8" t="s">
         <v>563</v>
       </c>
       <c r="K80" s="1" t="s">
@@ -5546,7 +5589,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>141</v>
       </c>
@@ -5570,7 +5613,7 @@
       <c r="I81" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J81" s="1" t="s">
+      <c r="J81" s="8" t="s">
         <v>564</v>
       </c>
       <c r="K81" s="1" t="s">
@@ -5583,7 +5626,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>164</v>
       </c>
@@ -5607,7 +5650,7 @@
       <c r="I82" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J82" s="1" t="s">
+      <c r="J82" s="8" t="s">
         <v>565</v>
       </c>
       <c r="K82" s="1" t="s">
@@ -5620,7 +5663,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>77</v>
       </c>
@@ -5648,7 +5691,7 @@
       <c r="I83" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J83" s="1" t="s">
+      <c r="J83" s="8" t="s">
         <v>566</v>
       </c>
       <c r="K83" s="1" t="s">
@@ -5689,7 +5732,7 @@
       <c r="I84" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J84" s="1" t="s">
+      <c r="J84" s="8" t="s">
         <v>568</v>
       </c>
       <c r="K84" s="1" t="s">
@@ -5730,7 +5773,7 @@
       <c r="I85" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J85" s="1" t="s">
+      <c r="J85" s="8" t="s">
         <v>569</v>
       </c>
       <c r="K85" s="1" t="s">
@@ -5771,8 +5814,8 @@
       <c r="I86" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J86" s="1" t="s">
-        <v>607</v>
+      <c r="J86" s="8" t="s">
+        <v>646</v>
       </c>
       <c r="K86" s="1" t="s">
         <v>21</v>
@@ -5812,7 +5855,7 @@
       <c r="I87" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J87" s="1" t="s">
+      <c r="J87" s="8" t="s">
         <v>570</v>
       </c>
       <c r="K87" s="1" t="s">
@@ -5853,8 +5896,8 @@
       <c r="I88" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J88" s="3" t="s">
-        <v>606</v>
+      <c r="J88" s="9" t="s">
+        <v>645</v>
       </c>
       <c r="K88" s="1" t="s">
         <v>21</v>
@@ -5894,7 +5937,7 @@
       <c r="I89" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J89" s="1" t="s">
+      <c r="J89" s="8" t="s">
         <v>571</v>
       </c>
       <c r="K89" s="1" t="s">
@@ -5931,8 +5974,8 @@
       <c r="I90" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J90" s="1" t="s">
-        <v>605</v>
+      <c r="J90" s="8" t="s">
+        <v>647</v>
       </c>
       <c r="K90" s="1" t="s">
         <v>21</v>
@@ -5972,7 +6015,7 @@
       <c r="I91" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J91" s="3" t="s">
+      <c r="J91" s="9" t="s">
         <v>597</v>
       </c>
       <c r="K91" s="1" t="s">
@@ -6009,7 +6052,7 @@
       <c r="I92" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J92" s="1" t="s">
+      <c r="J92" s="8" t="s">
         <v>572</v>
       </c>
       <c r="K92" s="1" t="s">
@@ -6046,7 +6089,7 @@
       <c r="I93" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J93" s="1" t="s">
+      <c r="J93" s="8" t="s">
         <v>573</v>
       </c>
       <c r="K93" s="1" t="s">
@@ -6087,7 +6130,7 @@
       <c r="I94" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J94" s="1" t="s">
+      <c r="J94" s="8" t="s">
         <v>574</v>
       </c>
       <c r="K94" s="1" t="s">
@@ -6128,7 +6171,7 @@
       <c r="I95" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J95" s="1" t="s">
+      <c r="J95" s="8" t="s">
         <v>567</v>
       </c>
       <c r="K95" s="1" t="s">
@@ -6169,7 +6212,7 @@
       <c r="I96" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J96" s="1" t="s">
+      <c r="J96" s="8" t="s">
         <v>575</v>
       </c>
       <c r="K96" s="1" t="s">
@@ -6182,7 +6225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>454</v>
       </c>
@@ -6206,7 +6249,7 @@
       <c r="I97" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J97" s="1" t="s">
+      <c r="J97" s="8" t="s">
         <v>576</v>
       </c>
       <c r="K97" s="1" t="s">
@@ -6219,7 +6262,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>200</v>
       </c>
@@ -6247,7 +6290,7 @@
       <c r="I98" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J98" s="1" t="s">
+      <c r="J98" s="8" t="s">
         <v>577</v>
       </c>
       <c r="K98" s="1" t="s">
@@ -6260,7 +6303,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>364</v>
       </c>
@@ -6284,7 +6327,7 @@
       <c r="I99" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J99" s="1" t="s">
+      <c r="J99" s="8" t="s">
         <v>578</v>
       </c>
       <c r="K99" s="1" t="s">
@@ -6297,7 +6340,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>297</v>
       </c>
@@ -6321,7 +6364,7 @@
       <c r="I100" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J100" s="1" t="s">
+      <c r="J100" s="8" t="s">
         <v>579</v>
       </c>
       <c r="K100" s="1" t="s">
@@ -6334,7 +6377,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>378</v>
       </c>
@@ -6358,7 +6401,7 @@
       <c r="I101" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J101" s="1" t="s">
+      <c r="J101" s="8" t="s">
         <v>580</v>
       </c>
       <c r="K101" s="1" t="s">
@@ -6371,7 +6414,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>167</v>
       </c>
@@ -6395,7 +6438,7 @@
       <c r="I102" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J102" s="1" t="s">
+      <c r="J102" s="8" t="s">
         <v>581</v>
       </c>
       <c r="K102" s="1" t="s">
@@ -6408,7 +6451,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>97</v>
       </c>
@@ -6436,7 +6479,7 @@
       <c r="I103" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J103" s="1" t="s">
+      <c r="J103" s="8" t="s">
         <v>582</v>
       </c>
       <c r="K103" s="1" t="s">
@@ -6449,7 +6492,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>127</v>
       </c>
@@ -6477,7 +6520,7 @@
       <c r="I104" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J104" s="1" t="s">
+      <c r="J104" s="8" t="s">
         <v>583</v>
       </c>
       <c r="K104" s="1" t="s">
@@ -6490,7 +6533,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>100</v>
       </c>
@@ -6518,7 +6561,7 @@
       <c r="I105" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J105" s="1" t="s">
+      <c r="J105" s="8" t="s">
         <v>584</v>
       </c>
       <c r="K105" s="1" t="s">
@@ -6559,7 +6602,7 @@
       <c r="I106" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J106" s="1" t="s">
+      <c r="J106" s="8" t="s">
         <v>586</v>
       </c>
       <c r="K106" s="1" t="s">
@@ -6572,7 +6615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>231</v>
       </c>
@@ -6600,7 +6643,7 @@
       <c r="I107" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J107" s="1" t="s">
+      <c r="J107" s="8" t="s">
         <v>585</v>
       </c>
       <c r="K107" s="1" t="s">
@@ -6613,7 +6656,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>195</v>
       </c>
@@ -6637,7 +6680,7 @@
       <c r="I108" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="J108" s="1" t="s">
+      <c r="J108" s="8" t="s">
         <v>587</v>
       </c>
       <c r="K108" s="1" t="s">
@@ -6650,7 +6693,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>353</v>
       </c>
@@ -6674,7 +6717,7 @@
       <c r="I109" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J109" s="1" t="s">
+      <c r="J109" s="8" t="s">
         <v>588</v>
       </c>
       <c r="K109" s="1" t="s">
@@ -6687,7 +6730,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>45</v>
       </c>
@@ -6715,7 +6758,7 @@
       <c r="I110" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J110" s="1" t="s">
+      <c r="J110" s="8" t="s">
         <v>539</v>
       </c>
       <c r="K110" s="1" t="s">
@@ -6728,7 +6771,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>173</v>
       </c>
@@ -6756,7 +6799,7 @@
       <c r="I111" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J111" s="1" t="s">
+      <c r="J111" s="8" t="s">
         <v>538</v>
       </c>
       <c r="K111" s="1" t="s">
@@ -6769,7 +6812,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>124</v>
       </c>
@@ -6797,7 +6840,7 @@
       <c r="I112" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J112" s="1" t="s">
+      <c r="J112" s="8" t="s">
         <v>537</v>
       </c>
       <c r="K112" s="1" t="s">
@@ -6810,7 +6853,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>53</v>
       </c>
@@ -6838,7 +6881,7 @@
       <c r="I113" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J113" s="1" t="s">
+      <c r="J113" s="8" t="s">
         <v>536</v>
       </c>
       <c r="K113" s="1" t="s">
@@ -6875,7 +6918,7 @@
       <c r="I114" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J114" s="1" t="s">
+      <c r="J114" s="8" t="s">
         <v>535</v>
       </c>
       <c r="K114" s="1" t="s">
@@ -6888,7 +6931,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>12</v>
       </c>
@@ -6916,7 +6959,7 @@
       <c r="I115" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J115" s="1" t="s">
+      <c r="J115" s="8" t="s">
         <v>534</v>
       </c>
       <c r="K115" s="1" t="s">
@@ -6929,7 +6972,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>181</v>
       </c>
@@ -6957,7 +7000,7 @@
       <c r="I116" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J116" s="1" t="s">
+      <c r="J116" s="8" t="s">
         <v>533</v>
       </c>
       <c r="K116" s="1" t="s">
@@ -6970,7 +7013,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>359</v>
       </c>
@@ -6994,7 +7037,7 @@
       <c r="I117" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J117" s="1" t="s">
+      <c r="J117" s="8" t="s">
         <v>532</v>
       </c>
       <c r="K117" s="1" t="s">
@@ -7007,7 +7050,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>170</v>
       </c>
@@ -7031,7 +7074,7 @@
       <c r="I118" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J118" s="1" t="s">
+      <c r="J118" s="8" t="s">
         <v>531</v>
       </c>
       <c r="K118" s="1" t="s">
@@ -7044,7 +7087,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>103</v>
       </c>
@@ -7072,7 +7115,7 @@
       <c r="I119" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J119" s="1" t="s">
+      <c r="J119" s="8" t="s">
         <v>530</v>
       </c>
       <c r="K119" s="1" t="s">
@@ -7085,7 +7128,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>288</v>
       </c>
@@ -7109,7 +7152,7 @@
       <c r="I120" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J120" s="1" t="s">
+      <c r="J120" s="8" t="s">
         <v>529</v>
       </c>
       <c r="K120" s="1" t="s">
@@ -7122,7 +7165,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>81</v>
       </c>
@@ -7150,7 +7193,7 @@
       <c r="I121" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J121" s="1" t="s">
+      <c r="J121" s="8" t="s">
         <v>527</v>
       </c>
       <c r="K121" s="1" t="s">
@@ -7163,7 +7206,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>86</v>
       </c>
@@ -7191,7 +7234,7 @@
       <c r="I122" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J122" s="1" t="s">
+      <c r="J122" s="8" t="s">
         <v>526</v>
       </c>
       <c r="K122" s="4" t="s">
@@ -7204,7 +7247,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="123" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:13" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>92</v>
       </c>
@@ -7232,7 +7275,7 @@
       <c r="I123" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J123" s="1" t="s">
+      <c r="J123" s="8" t="s">
         <v>525</v>
       </c>
       <c r="K123" s="1" t="s">
@@ -7245,7 +7288,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
         <v>74</v>
       </c>
@@ -7273,7 +7316,7 @@
       <c r="I124" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J124" s="5" t="s">
+      <c r="J124" s="10" t="s">
         <v>528</v>
       </c>
       <c r="K124" s="5" t="s">
@@ -7286,7 +7329,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>106</v>
       </c>
@@ -7314,7 +7357,7 @@
       <c r="I125" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J125" s="1" t="s">
+      <c r="J125" s="8" t="s">
         <v>524</v>
       </c>
       <c r="K125" s="1" t="s">
@@ -7327,7 +7370,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>109</v>
       </c>
@@ -7355,7 +7398,7 @@
       <c r="I126" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J126" s="1" t="s">
+      <c r="J126" s="8" t="s">
         <v>523</v>
       </c>
       <c r="K126" s="1" t="s">
@@ -7368,7 +7411,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>112</v>
       </c>
@@ -7396,7 +7439,7 @@
       <c r="I127" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J127" s="1" t="s">
+      <c r="J127" s="8" t="s">
         <v>522</v>
       </c>
       <c r="K127" s="1" t="s">
@@ -7409,7 +7452,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>303</v>
       </c>
@@ -7433,7 +7476,7 @@
       <c r="I128" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J128" s="1" t="s">
+      <c r="J128" s="8" t="s">
         <v>521</v>
       </c>
       <c r="K128" s="1" t="s">
@@ -7446,7 +7489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>32</v>
       </c>
@@ -7474,7 +7517,7 @@
       <c r="I129" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J129" s="1" t="s">
+      <c r="J129" s="8" t="s">
         <v>590</v>
       </c>
       <c r="K129" s="1" t="s">
@@ -7487,7 +7530,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>32</v>
       </c>
@@ -7515,7 +7558,7 @@
       <c r="I130" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J130" s="1" t="s">
+      <c r="J130" s="8" t="s">
         <v>520</v>
       </c>
       <c r="K130" s="1" t="s">
@@ -7528,36 +7571,36 @@
         <v>23</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>608</v>
+        <v>34</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>15</v>
+        <v>605</v>
       </c>
       <c r="E131" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>17</v>
+        <v>606</v>
       </c>
       <c r="G131" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H131" s="1" t="s">
-        <v>19</v>
+        <v>607</v>
       </c>
       <c r="I131" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J131" s="1" t="s">
-        <v>621</v>
+      <c r="J131" s="8" t="s">
+        <v>637</v>
       </c>
       <c r="K131" s="1" t="s">
         <v>21</v>
@@ -7566,39 +7609,39 @@
         <v>22</v>
       </c>
       <c r="M131" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C132" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D132" s="1" t="s">
         <v>609</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="E132" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>17</v>
+        <v>610</v>
       </c>
       <c r="G132" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H132" s="1" t="s">
-        <v>19</v>
+        <v>611</v>
       </c>
       <c r="I132" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J132" s="1" t="s">
-        <v>622</v>
+      <c r="J132" s="8" t="s">
+        <v>638</v>
       </c>
       <c r="K132" s="1" t="s">
         <v>21</v>
@@ -7607,39 +7650,39 @@
         <v>22</v>
       </c>
       <c r="M132" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="133" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B133" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>610</v>
+        <v>34</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>15</v>
+        <v>613</v>
       </c>
       <c r="E133" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>17</v>
+        <v>614</v>
       </c>
       <c r="G133" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H133" s="1" t="s">
-        <v>19</v>
+        <v>615</v>
       </c>
       <c r="I133" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J133" s="1" t="s">
-        <v>623</v>
+      <c r="J133" s="8" t="s">
+        <v>639</v>
       </c>
       <c r="K133" s="1" t="s">
         <v>21</v>
@@ -7648,39 +7691,39 @@
         <v>22</v>
       </c>
       <c r="M133" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="134" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>611</v>
+        <v>34</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>15</v>
+        <v>617</v>
       </c>
       <c r="E134" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>17</v>
+        <v>618</v>
       </c>
       <c r="G134" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H134" s="1" t="s">
-        <v>19</v>
+        <v>619</v>
       </c>
       <c r="I134" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J134" s="1" t="s">
-        <v>612</v>
+      <c r="J134" s="8" t="s">
+        <v>640</v>
       </c>
       <c r="K134" s="1" t="s">
         <v>21</v>
@@ -7689,80 +7732,80 @@
         <v>22</v>
       </c>
       <c r="M134" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="135" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>613</v>
+        <v>34</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>15</v>
+        <v>621</v>
       </c>
       <c r="E135" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>17</v>
+        <v>622</v>
       </c>
       <c r="G135" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>19</v>
+        <v>623</v>
       </c>
       <c r="I135" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J135" s="1" t="s">
+      <c r="J135" s="8" t="s">
+        <v>641</v>
+      </c>
+      <c r="K135" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L135" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M135" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="K135" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L135" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M135" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="136" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>614</v>
+        <v>34</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>15</v>
+        <v>625</v>
       </c>
       <c r="E136" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>17</v>
+        <v>626</v>
       </c>
       <c r="G136" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H136" s="1" t="s">
-        <v>19</v>
+        <v>627</v>
       </c>
       <c r="I136" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J136" s="1" t="s">
-        <v>625</v>
+      <c r="J136" s="8" t="s">
+        <v>642</v>
       </c>
       <c r="K136" s="1" t="s">
         <v>21</v>
@@ -7771,39 +7814,39 @@
         <v>22</v>
       </c>
       <c r="M136" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="137" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>615</v>
+        <v>34</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>15</v>
+        <v>629</v>
       </c>
       <c r="E137" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F137" s="1" t="s">
-        <v>17</v>
+        <v>630</v>
       </c>
       <c r="G137" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>19</v>
+        <v>631</v>
       </c>
       <c r="I137" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J137" s="1" t="s">
-        <v>626</v>
+      <c r="J137" s="8" t="s">
+        <v>643</v>
       </c>
       <c r="K137" s="1" t="s">
         <v>21</v>
@@ -7812,39 +7855,39 @@
         <v>22</v>
       </c>
       <c r="M137" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="138" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>616</v>
+        <v>34</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>15</v>
+        <v>633</v>
       </c>
       <c r="E138" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F138" s="1" t="s">
-        <v>17</v>
+        <v>634</v>
       </c>
       <c r="G138" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>19</v>
+        <v>635</v>
       </c>
       <c r="I138" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J138" s="1" t="s">
-        <v>627</v>
+      <c r="J138" s="8" t="s">
+        <v>644</v>
       </c>
       <c r="K138" s="1" t="s">
         <v>21</v>
@@ -7853,175 +7896,16 @@
         <v>22</v>
       </c>
       <c r="M138" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A139" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B139" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C139" s="7" t="s">
-        <v>617</v>
-      </c>
-      <c r="D139" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E139" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F139" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G139" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H139" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I139" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J139" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="K139" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L139" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M139" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A140" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B140" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>618</v>
-      </c>
-      <c r="D140" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F140" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G140" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H140" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I140" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J140" s="1" t="s">
-        <v>628</v>
-      </c>
-      <c r="K140" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L140" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M140" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A141" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B141" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C141" s="1" t="s">
-        <v>619</v>
-      </c>
-      <c r="D141" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E141" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F141" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G141" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H141" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I141" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J141" s="1" t="s">
-        <v>630</v>
-      </c>
-      <c r="K141" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L141" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M141" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A142" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B142" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C142" s="1" t="s">
-        <v>620</v>
-      </c>
-      <c r="D142" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E142" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F142" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G142" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H142" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I142" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J142" s="1" t="s">
-        <v>629</v>
-      </c>
-      <c r="K142" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L142" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M142" s="1" t="s">
-        <v>23</v>
+        <v>636</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M142" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:M138" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="GRD00001"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M130">
       <sortCondition ref="J1:J130"/>
     </sortState>
@@ -8029,20 +7913,15 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M116">
     <sortCondition ref="C1:C116"/>
   </sortState>
-  <conditionalFormatting sqref="C140:C142 C131:C138">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="C1:C126">
+    <cfRule type="duplicateValues" dxfId="2" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C143:C1048576 C1:C126">
-    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+  <conditionalFormatting sqref="C127:C138">
+    <cfRule type="duplicateValues" dxfId="1" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J131:J142">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J143:J1048576 J1:J130">
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C127:C130">
-    <cfRule type="duplicateValues" dxfId="0" priority="39"/>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>